<commit_message>
📊 Actualizar VENTAS_Y_ABONOS_VU.xlsx — 14-04-2026, 2:01:51 p. m.
</commit_message>
<xml_diff>
--- a/datos/VENTAS_Y_ABONOS_VU.xlsx
+++ b/datos/VENTAS_Y_ABONOS_VU.xlsx
@@ -5,22 +5,35 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/abril/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E863AA2B-CC16-4145-A384-3A16DA2255F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0EC2351E-B038-4787-A2C6-39629E12774D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ParamQuery Pro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="290">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -142,108 +155,351 @@
     <t>VALLES UNIDOS S.A.</t>
   </si>
   <si>
-    <t>1015744</t>
+    <t>1015779</t>
+  </si>
+  <si>
+    <t>ABONADO</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>GERENCIA NECESIDAD FUTURA TERRENO</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Camilo Jesus Medel Rojas</t>
+  </si>
+  <si>
+    <t>daniela castro valdebenito</t>
+  </si>
+  <si>
+    <t>VENEGAS ASTORGA IRIS DEL CARMEN</t>
+  </si>
+  <si>
+    <t>11739202-3</t>
+  </si>
+  <si>
+    <t>Los espinos , ALT 138 - Lampa -</t>
+  </si>
+  <si>
+    <t>Metropolitana</t>
+  </si>
+  <si>
+    <t>Chacabuco</t>
+  </si>
+  <si>
+    <t>Lampa</t>
+  </si>
+  <si>
+    <t>931276144 - 56931276144</t>
+  </si>
+  <si>
+    <t>irisvenegas260@gmail.com - IRISVENEGAS260@GMAIL.CO</t>
+  </si>
+  <si>
+    <t>Mantención Perpetua Simple</t>
+  </si>
+  <si>
+    <t>PESOS</t>
+  </si>
+  <si>
+    <t>4600000</t>
+  </si>
+  <si>
+    <t>414000</t>
+  </si>
+  <si>
+    <t>0.09</t>
+  </si>
+  <si>
+    <t>460000</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>4140000</t>
+  </si>
+  <si>
+    <t>3478991.597</t>
+  </si>
+  <si>
+    <t>3726000</t>
+  </si>
+  <si>
+    <t>OFICINA</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>155250</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>05/05/2026</t>
+  </si>
+  <si>
+    <t>2026-02-12T00:00:00</t>
+  </si>
+  <si>
+    <t>1015785</t>
   </si>
   <si>
     <t>COMPLETADO</t>
   </si>
   <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>GERENCIA NECESIDAD FUTURA TERRENO</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Camilo Jesus Medel Rojas</t>
-  </si>
-  <si>
-    <t>daniela castro valdebenito</t>
-  </si>
-  <si>
-    <t>VENEGAS ASTORGA IRIS DEL CARMEN</t>
-  </si>
-  <si>
-    <t>11739202-3</t>
-  </si>
-  <si>
-    <t>Los espinos , ALT 138 - Lampa -</t>
-  </si>
-  <si>
-    <t>Metropolitana</t>
-  </si>
-  <si>
-    <t>Chacabuco</t>
-  </si>
-  <si>
-    <t>Lampa</t>
-  </si>
-  <si>
-    <t>931276144 - 56931276144</t>
-  </si>
-  <si>
-    <t>irisvenegas260@gmail.com - IRISVENEGAS260@GMAIL.CO</t>
-  </si>
-  <si>
-    <t>Mantención Perpetua Simple</t>
-  </si>
-  <si>
-    <t>PESOS</t>
-  </si>
-  <si>
-    <t>4600000</t>
-  </si>
-  <si>
-    <t>414000</t>
-  </si>
-  <si>
-    <t>0.09</t>
-  </si>
-  <si>
-    <t>460000</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>4140000</t>
-  </si>
-  <si>
-    <t>3478991.597</t>
-  </si>
-  <si>
-    <t>3726000</t>
-  </si>
-  <si>
-    <t>OFICINA</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>155250</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>05/05/2026</t>
-  </si>
-  <si>
-    <t>2026-02-12T00:00:00</t>
+    <t>Luis Alberto Osores Osores</t>
+  </si>
+  <si>
+    <t>CHAVEZ QUILODRAN SERGIO ENRIQUE</t>
+  </si>
+  <si>
+    <t>9278099-6</t>
+  </si>
+  <si>
+    <t>Pasaje vivaldi , ALT 156 - Quilicura -</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Quilicura</t>
+  </si>
+  <si>
+    <t>942897680</t>
+  </si>
+  <si>
+    <t>kekochavezquilodran@gmail.com</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>93150</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>09/05/2026</t>
+  </si>
+  <si>
+    <t>2026-04-10T00:00:00</t>
+  </si>
+  <si>
+    <t>1015783</t>
+  </si>
+  <si>
+    <t>300000</t>
+  </si>
+  <si>
+    <t>GABRIELA DEL CARMEN ROJAS QUEZADA</t>
+  </si>
+  <si>
+    <t>Yohany Margarita Gonzalez Rojas</t>
+  </si>
+  <si>
+    <t>JORQUERA VALENZUELA EMMA ROSA</t>
+  </si>
+  <si>
+    <t>67384547</t>
+  </si>
+  <si>
+    <t>Carlos dittborn, ALT 95 - Quilicura -</t>
+  </si>
+  <si>
+    <t>973382698 - +56973382698</t>
+  </si>
+  <si>
+    <t>emmajorquera2@gmail.com</t>
+  </si>
+  <si>
+    <t>Mantención Perpetua Integral</t>
+  </si>
+  <si>
+    <t>3000000</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>2700000</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>37500</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>13/05/2026</t>
+  </si>
+  <si>
+    <t>2026-04-13T00:00:00</t>
+  </si>
+  <si>
+    <t>1015764</t>
+  </si>
+  <si>
+    <t>Marcela Antonia  Valdés  Barrios</t>
+  </si>
+  <si>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>ALVARADO ORTIZ JACQUELINE DEL CARMEN</t>
+  </si>
+  <si>
+    <t>9765730-0</t>
+  </si>
+  <si>
+    <t>ALFREDO SANTANDER 1539, Quilicura, Santiago, Metropolitana  Casa:</t>
+  </si>
+  <si>
+    <t>988574499</t>
+  </si>
+  <si>
+    <t>jacquelinealvarado356@gmail.com</t>
+  </si>
+  <si>
+    <t>2521008.4</t>
+  </si>
+  <si>
+    <t>112500</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>19/05/2026</t>
+  </si>
+  <si>
+    <t>1015766</t>
+  </si>
+  <si>
+    <t>Rodrigo Ignacio Castro Figueroa</t>
+  </si>
+  <si>
+    <t>DOMINGUEZ BARRIOS MARTA ORIANA</t>
+  </si>
+  <si>
+    <t>7078549-8</t>
+  </si>
+  <si>
+    <t>Psj ventana, ALT 521 - Quilicura -</t>
+  </si>
+  <si>
+    <t>987185292</t>
+  </si>
+  <si>
+    <t>223515177</t>
+  </si>
+  <si>
+    <t>martadominguezbarrios@gmail.com</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>75000</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>20/05/2026</t>
+  </si>
+  <si>
+    <t>1015780</t>
+  </si>
+  <si>
+    <t>300079.52</t>
+  </si>
+  <si>
+    <t>NF CARTERA</t>
+  </si>
+  <si>
+    <t>FLORES AEDO VALERIA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>12512126-8</t>
+  </si>
+  <si>
+    <t>PJE OLLAGUE BLOK 251 DPT A-31, ALT 31 - LO MARCOLETA -</t>
+  </si>
+  <si>
+    <t>SANTIAGO</t>
+  </si>
+  <si>
+    <t>QUILICURA</t>
+  </si>
+  <si>
+    <t>LO MARCOLETA</t>
+  </si>
+  <si>
+    <t>965115499</t>
+  </si>
+  <si>
+    <t>D4075473@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>Planes Parque</t>
+  </si>
+  <si>
+    <t>Valle De La Memoria (cuotas)</t>
+  </si>
+  <si>
+    <t>Valle De La Memoria</t>
+  </si>
+  <si>
+    <t>4990000</t>
+  </si>
+  <si>
+    <t>2986395</t>
+  </si>
+  <si>
+    <t>59.85</t>
+  </si>
+  <si>
+    <t>2003605</t>
+  </si>
+  <si>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>3-AJ-41</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria</t>
+  </si>
+  <si>
+    <t>2023-07-31T00:00:00</t>
+  </si>
+  <si>
+    <t>1015781</t>
+  </si>
+  <si>
+    <t>105451</t>
   </si>
   <si>
     <t>1015755</t>
   </si>
   <si>
-    <t>82920</t>
-  </si>
-  <si>
-    <t>NF CARTERA</t>
-  </si>
-  <si>
     <t>07/04/2026</t>
   </si>
   <si>
@@ -262,24 +518,6 @@
     <t>yvanaparada71@gmail.com</t>
   </si>
   <si>
-    <t>Planes Parque</t>
-  </si>
-  <si>
-    <t>Valle De La Memoria (cuotas)</t>
-  </si>
-  <si>
-    <t>Valle De La Memoria</t>
-  </si>
-  <si>
-    <t>4990000</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>3000000</t>
-  </si>
-  <si>
     <t>60.12</t>
   </si>
   <si>
@@ -295,22 +533,274 @@
     <t>07/05/2026</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>3-AM-25</t>
   </si>
   <si>
-    <t>Valle de la Memoria</t>
-  </si>
-  <si>
     <t>2026-03-26T00:00:00</t>
   </si>
   <si>
+    <t>1015782</t>
+  </si>
+  <si>
+    <t>350000</t>
+  </si>
+  <si>
+    <t>MUÑOZ PEÑA CLAUDIO GREGORIO</t>
+  </si>
+  <si>
+    <t>12834568-K</t>
+  </si>
+  <si>
+    <t>RIO MAULE 2750 CASA 85, ALT 85 - VALLE GRANDE -</t>
+  </si>
+  <si>
+    <t>LAMPA</t>
+  </si>
+  <si>
+    <t>VALLE GRANDE</t>
+  </si>
+  <si>
+    <t>974526722</t>
+  </si>
+  <si>
+    <t>4220000</t>
+  </si>
+  <si>
+    <t>84.57</t>
+  </si>
+  <si>
+    <t>770000</t>
+  </si>
+  <si>
+    <t>154000</t>
+  </si>
+  <si>
+    <t>3-M-24</t>
+  </si>
+  <si>
+    <t>2026-04-09T00:00:00</t>
+  </si>
+  <si>
+    <t>1015786</t>
+  </si>
+  <si>
+    <t>1360000</t>
+  </si>
+  <si>
+    <t>Fernanda Scarlet Cuevas Olivares</t>
+  </si>
+  <si>
+    <t>CARVAJAL SAGREDO RAFAEL IGNACIO</t>
+  </si>
+  <si>
+    <t>9867041-6</t>
+  </si>
+  <si>
+    <t>Las pablonias, ALT 1485 - Quilicura -</t>
+  </si>
+  <si>
+    <t>966273118</t>
+  </si>
+  <si>
+    <t>rafael.sagredo@gmail.com</t>
+  </si>
+  <si>
+    <t>Planes Descanso de Cenizas</t>
+  </si>
+  <si>
+    <t>Destellos De Luz</t>
+  </si>
+  <si>
+    <t>Destellos de Luz</t>
+  </si>
+  <si>
+    <t>1700000</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>340000</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>14/05/2026</t>
+  </si>
+  <si>
+    <t>SIN ASIGNAR</t>
+  </si>
+  <si>
+    <t>MIGRAR</t>
+  </si>
+  <si>
+    <t>2026-04-14T00:00:00</t>
+  </si>
+  <si>
+    <t>1015758</t>
+  </si>
+  <si>
+    <t>ERNESTO OLIVA</t>
+  </si>
+  <si>
+    <t>MIGUEL SANDOVAL</t>
+  </si>
+  <si>
+    <t>ANDREA CONCHA ADASME</t>
+  </si>
+  <si>
+    <t>MUÑOZ FLORES MANUEL  ALEJANDRO</t>
+  </si>
+  <si>
+    <t>12112040-3</t>
+  </si>
+  <si>
+    <t>Las petunias  540, Quilicura, Santiago, Metropolitana  Casa:</t>
+  </si>
+  <si>
+    <t>921609666</t>
+  </si>
+  <si>
+    <t>martha.moontero@hotmail.com</t>
+  </si>
+  <si>
+    <t>500000</t>
+  </si>
+  <si>
+    <t>499000</t>
+  </si>
+  <si>
+    <t>4491000</t>
+  </si>
+  <si>
+    <t>3991000</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>66497</t>
+  </si>
+  <si>
+    <t>3-BD-34</t>
+  </si>
+  <si>
+    <t>1015735</t>
+  </si>
+  <si>
+    <t>LIDIA MONICA FLORES BRAVO</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>ROBLES CISTERNAS MARGARITA ALEJANDRA</t>
+  </si>
+  <si>
+    <t>12353329-1</t>
+  </si>
+  <si>
+    <t>El medio dia, ALT 358 - Quilicura -</t>
+  </si>
+  <si>
+    <t>994485350</t>
+  </si>
+  <si>
+    <t>robles.cisterm@gmail.com</t>
+  </si>
+  <si>
+    <t>4490000</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>76084</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>15/05/2026</t>
+  </si>
+  <si>
+    <t>3-V-21</t>
+  </si>
+  <si>
+    <t>1015750</t>
+  </si>
+  <si>
+    <t>08/04/2026</t>
+  </si>
+  <si>
+    <t>SANCHEZ MATUS ISAAC  ESTEBAN</t>
+  </si>
+  <si>
+    <t>17517932-1</t>
+  </si>
+  <si>
+    <t>Blanco encalada  102, Quilicura, Santiago, Metropolitana  Pi/dp Casa E Casa:</t>
+  </si>
+  <si>
+    <t>984602304</t>
+  </si>
+  <si>
+    <t>930860950</t>
+  </si>
+  <si>
+    <t>aylenyanto23@gmail.com</t>
+  </si>
+  <si>
+    <t>4-A-27</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria 2</t>
+  </si>
+  <si>
+    <t>1015748</t>
+  </si>
+  <si>
+    <t>Estefany francisca gonzalez morales</t>
+  </si>
+  <si>
+    <t>YASMELY RAMONA VARGAS INFANTE</t>
+  </si>
+  <si>
+    <t>VARGAS CAMPOS LUIS MIGUEL</t>
+  </si>
+  <si>
+    <t>12003266-6</t>
+  </si>
+  <si>
+    <t>Blanco Encalada, ALT 144 - Quilicura -</t>
+  </si>
+  <si>
+    <t>931377299</t>
+  </si>
+  <si>
+    <t>LUISMIGUEL.VARGASC@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>450000</t>
+  </si>
+  <si>
+    <t>4041000</t>
+  </si>
+  <si>
+    <t>112250</t>
+  </si>
+  <si>
+    <t>4-O-25</t>
+  </si>
+  <si>
     <t>1015757</t>
   </si>
   <si>
-    <t>350000</t>
+    <t>13/04/2026</t>
   </si>
   <si>
     <t>VARGAS AGUIRRE CARLOS ANTONIO</t>
@@ -322,12 +812,6 @@
     <t>PUCON 409, ALT 409 - Quilicura -</t>
   </si>
   <si>
-    <t>Santiago</t>
-  </si>
-  <si>
-    <t>Quilicura</t>
-  </si>
-  <si>
     <t>985674375</t>
   </si>
   <si>
@@ -346,10 +830,7 @@
     <t>3445000</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>57416.66</t>
+    <t>57397</t>
   </si>
   <si>
     <t>30</t>
@@ -361,247 +842,7 @@
     <t>4-Z-39</t>
   </si>
   <si>
-    <t>Valle de la Memoria 2</t>
-  </si>
-  <si>
     <t>2026-04-01T00:00:00</t>
-  </si>
-  <si>
-    <t>1015752</t>
-  </si>
-  <si>
-    <t>ABONADO</t>
-  </si>
-  <si>
-    <t>300000</t>
-  </si>
-  <si>
-    <t>Rodrigo Ignacio Castro Figueroa</t>
-  </si>
-  <si>
-    <t>DOMINGUEZ BARRIOS MARTA ORIANA</t>
-  </si>
-  <si>
-    <t>7078549-8</t>
-  </si>
-  <si>
-    <t>Psj ventana, ALT 521 - Quilicura -</t>
-  </si>
-  <si>
-    <t>987185292</t>
-  </si>
-  <si>
-    <t>223515177</t>
-  </si>
-  <si>
-    <t>martadominguezbarrios@gmail.com</t>
-  </si>
-  <si>
-    <t>Mantención Perpetua Integral</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
-    <t>2700000</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>75000</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>20/05/2026</t>
-  </si>
-  <si>
-    <t>2026-04-06T00:00:00</t>
-  </si>
-  <si>
-    <t>1015739</t>
-  </si>
-  <si>
-    <t>Marcela Antonia  Valdés  Barrios</t>
-  </si>
-  <si>
-    <t>ALVARADO ORTIZ ORTIZ JACQUELINE DEL CARMEN</t>
-  </si>
-  <si>
-    <t>9765730-0</t>
-  </si>
-  <si>
-    <t>ALFREDO SANTANDER, ALT 1539 - Quilicura -</t>
-  </si>
-  <si>
-    <t>988574499</t>
-  </si>
-  <si>
-    <t>jacquelinealvarado356@gmail.com</t>
-  </si>
-  <si>
-    <t>112500</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>19/05/2026</t>
-  </si>
-  <si>
-    <t>2026-04-07T00:00:00</t>
-  </si>
-  <si>
-    <t>1015758</t>
-  </si>
-  <si>
-    <t>500000</t>
-  </si>
-  <si>
-    <t>ERNESTO OLIVA</t>
-  </si>
-  <si>
-    <t>MIGUEL SANDOVAL</t>
-  </si>
-  <si>
-    <t>ANDREA CONCHA ADASME</t>
-  </si>
-  <si>
-    <t>MUÑOZ FLORES MANUEL ALEJANDRO</t>
-  </si>
-  <si>
-    <t>12.112.040-3</t>
-  </si>
-  <si>
-    <t>Las petunias , ALT 540 - Quilicura -</t>
-  </si>
-  <si>
-    <t>921609666</t>
-  </si>
-  <si>
-    <t>martha.moontero@hotmail.com</t>
-  </si>
-  <si>
-    <t>499000</t>
-  </si>
-  <si>
-    <t>4491000</t>
-  </si>
-  <si>
-    <t>3991000</t>
-  </si>
-  <si>
-    <t>66516.66</t>
-  </si>
-  <si>
-    <t>3-BD-34</t>
-  </si>
-  <si>
-    <t>1015735</t>
-  </si>
-  <si>
-    <t>GABRIELA DEL CARMEN ROJAS QUEZADA</t>
-  </si>
-  <si>
-    <t>LIDIA MONICA FLORES BRAVO</t>
-  </si>
-  <si>
-    <t>31/03/2026</t>
-  </si>
-  <si>
-    <t>ROBLES CISTERNAS MARGARITA ALEJANDRA</t>
-  </si>
-  <si>
-    <t>12353329-1</t>
-  </si>
-  <si>
-    <t>El medio dia, ALT 358 - Quilicura -</t>
-  </si>
-  <si>
-    <t>994485350</t>
-  </si>
-  <si>
-    <t>robles.cisterm@gmail.com</t>
-  </si>
-  <si>
-    <t>4490000</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>76084</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>15/05/2026</t>
-  </si>
-  <si>
-    <t>3-V-21</t>
-  </si>
-  <si>
-    <t>1015750</t>
-  </si>
-  <si>
-    <t>SANCHEZ MATUS ISAAC  ESTEBAN</t>
-  </si>
-  <si>
-    <t>17517932-1</t>
-  </si>
-  <si>
-    <t>Blanco encalada  102, Quilicura, Santiago, Metropolitana  Pi/dp Casa E Casa:</t>
-  </si>
-  <si>
-    <t>984602304</t>
-  </si>
-  <si>
-    <t>930860950</t>
-  </si>
-  <si>
-    <t>aylenyanto23@gmail.com</t>
-  </si>
-  <si>
-    <t>4-A-27</t>
-  </si>
-  <si>
-    <t>1015748</t>
-  </si>
-  <si>
-    <t>Estefany francisca gonzalez morales</t>
-  </si>
-  <si>
-    <t>YASMELY RAMONA VARGAS INFANTE</t>
-  </si>
-  <si>
-    <t>VARGAS CAMPOS LUIS MIGUEL</t>
-  </si>
-  <si>
-    <t>12003266-6</t>
-  </si>
-  <si>
-    <t>Blanco Encalada, ALT 144 - Quilicura -</t>
-  </si>
-  <si>
-    <t>931377299</t>
-  </si>
-  <si>
-    <t>LUISMIGUEL.VARGASC@GMAIL.COM</t>
-  </si>
-  <si>
-    <t>450000</t>
-  </si>
-  <si>
-    <t>4041000</t>
-  </si>
-  <si>
-    <t>112250</t>
-  </si>
-  <si>
-    <t>4-O-25</t>
   </si>
   <si>
     <t>1015754</t>
@@ -1522,11 +1763,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM11"/>
+  <dimension ref="A1:AM17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="38" width="8" customWidth="1"/>
-    <col min="39" max="39" width="15" customWidth="1"/>
+    <col min="1" max="39" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" x14ac:dyDescent="0.3">
@@ -1775,115 +2015,115 @@
         <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
         <v>44</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
         <v>73</v>
       </c>
       <c r="I3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" t="s">
         <v>74</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>75</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>76</v>
-      </c>
-      <c r="L3" t="s">
-        <v>77</v>
       </c>
       <c r="M3" t="s">
         <v>50</v>
       </c>
       <c r="N3" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="O3" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="P3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="S3" t="s">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="T3" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="U3" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="V3" t="s">
         <v>56</v>
       </c>
       <c r="W3" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="X3" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="Y3" t="s">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="Z3" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="AA3" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="AB3" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="AC3" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="AD3" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="AE3" t="s">
         <v>65</v>
       </c>
       <c r="AF3" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="AG3" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="AH3" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="AI3" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="AJ3" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="AK3" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="AL3" t="s">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="AM3" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.3">
@@ -1891,118 +2131,118 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
         <v>44</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="I4" t="s">
         <v>44</v>
       </c>
       <c r="J4" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="K4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="L4" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="M4" t="s">
         <v>50</v>
       </c>
       <c r="N4" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="O4" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="P4" t="s">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="Q4" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="R4" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="S4" t="s">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="T4" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="U4" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="V4" t="s">
         <v>56</v>
       </c>
       <c r="W4" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="X4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="Y4" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="Z4" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="AA4" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="AB4" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="AC4" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="AD4" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="AE4" t="s">
         <v>65</v>
       </c>
       <c r="AF4" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="AG4" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="AH4" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="AI4" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="AJ4" t="s">
-        <v>91</v>
+        <v>44</v>
       </c>
       <c r="AK4" t="s">
-        <v>112</v>
+        <v>44</v>
       </c>
       <c r="AL4" t="s">
-        <v>113</v>
+        <v>44</v>
       </c>
       <c r="AM4" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.3">
@@ -2010,13 +2250,13 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
         <v>43</v>
@@ -2028,88 +2268,88 @@
         <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="I5" t="s">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="J5" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="K5" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="L5" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="M5" t="s">
         <v>50</v>
       </c>
       <c r="N5" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="O5" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="P5" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="Q5" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="R5" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="S5" t="s">
         <v>44</v>
       </c>
       <c r="T5" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="U5" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="V5" t="s">
         <v>56</v>
       </c>
       <c r="W5" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="X5" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="Y5" t="s">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="Z5" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="AA5" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="AB5" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="AC5" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="AD5" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="AE5" t="s">
         <v>65</v>
       </c>
       <c r="AF5" t="s">
-        <v>128</v>
+        <v>66</v>
       </c>
       <c r="AG5" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="AH5" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="AI5" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="AJ5" t="s">
         <v>44</v>
@@ -2121,7 +2361,7 @@
         <v>44</v>
       </c>
       <c r="AM5" t="s">
-        <v>132</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.3">
@@ -2129,13 +2369,13 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
         <v>43</v>
@@ -2147,88 +2387,88 @@
         <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="I6" t="s">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="J6" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="K6" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="L6" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="M6" t="s">
         <v>50</v>
       </c>
       <c r="N6" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="O6" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="P6" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="Q6" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="R6" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="S6" t="s">
         <v>44</v>
       </c>
       <c r="T6" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="U6" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="V6" t="s">
         <v>56</v>
       </c>
       <c r="W6" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="X6" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="Y6" t="s">
-        <v>126</v>
+        <v>97</v>
       </c>
       <c r="Z6" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="AA6" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="AB6" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="AC6" t="s">
-        <v>85</v>
+        <v>113</v>
       </c>
       <c r="AD6" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="AE6" t="s">
         <v>65</v>
       </c>
       <c r="AF6" t="s">
-        <v>66</v>
+        <v>125</v>
       </c>
       <c r="AG6" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="AH6" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="AI6" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="AJ6" t="s">
         <v>44</v>
@@ -2240,7 +2480,7 @@
         <v>44</v>
       </c>
       <c r="AM6" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.3">
@@ -2248,118 +2488,118 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>146</v>
+        <v>44</v>
       </c>
       <c r="F7" t="s">
-        <v>146</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>147</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="I7" t="s">
         <v>44</v>
       </c>
       <c r="J7" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="K7" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="L7" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="M7" t="s">
-        <v>50</v>
+        <v>135</v>
       </c>
       <c r="N7" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="O7" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="P7" t="s">
-        <v>44</v>
+        <v>138</v>
       </c>
       <c r="Q7" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="R7" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="S7" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="T7" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="U7" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="V7" t="s">
         <v>56</v>
       </c>
       <c r="W7" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="X7" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>144</v>
+      </c>
+      <c r="AA7" t="s">
         <v>145</v>
       </c>
-      <c r="Y7" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>154</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>61</v>
-      </c>
       <c r="AB7" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="AC7" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="AD7" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="AE7" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="AF7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AG7" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="AH7" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="AI7" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="AJ7" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="AK7" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="AL7" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="AM7" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.3">
@@ -2367,118 +2607,118 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F8" t="s">
         <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>160</v>
+        <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="I8" t="s">
-        <v>162</v>
+        <v>107</v>
       </c>
       <c r="J8" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="L8" t="s">
-        <v>165</v>
+        <v>134</v>
       </c>
       <c r="M8" t="s">
-        <v>50</v>
+        <v>135</v>
       </c>
       <c r="N8" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="O8" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="P8" t="s">
-        <v>44</v>
+        <v>138</v>
       </c>
       <c r="Q8" t="s">
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="R8" t="s">
-        <v>167</v>
+        <v>139</v>
       </c>
       <c r="S8" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="T8" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="U8" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="V8" t="s">
         <v>56</v>
       </c>
       <c r="W8" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="X8" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>144</v>
+      </c>
+      <c r="AA8" t="s">
         <v>145</v>
       </c>
-      <c r="Y8" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>84</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>84</v>
-      </c>
       <c r="AB8" t="s">
-        <v>83</v>
+        <v>146</v>
       </c>
       <c r="AC8" t="s">
-        <v>83</v>
+        <v>146</v>
       </c>
       <c r="AD8" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
       <c r="AE8" t="s">
         <v>65</v>
       </c>
       <c r="AF8" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="AG8" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
       <c r="AH8" t="s">
-        <v>171</v>
+        <v>102</v>
       </c>
       <c r="AI8" t="s">
-        <v>172</v>
+        <v>103</v>
       </c>
       <c r="AJ8" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="AK8" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="AL8" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="AM8" t="s">
-        <v>44</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.3">
@@ -2486,118 +2726,118 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E9" t="s">
-        <v>146</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>146</v>
+        <v>44</v>
       </c>
       <c r="G9" t="s">
-        <v>147</v>
+        <v>44</v>
       </c>
       <c r="H9" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="I9" t="s">
-        <v>44</v>
+        <v>155</v>
       </c>
       <c r="J9" t="s">
-        <v>175</v>
+        <v>156</v>
       </c>
       <c r="K9" t="s">
-        <v>176</v>
+        <v>157</v>
       </c>
       <c r="L9" t="s">
-        <v>177</v>
+        <v>158</v>
       </c>
       <c r="M9" t="s">
         <v>50</v>
       </c>
       <c r="N9" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="O9" t="s">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="P9" t="s">
-        <v>178</v>
+        <v>159</v>
       </c>
       <c r="Q9" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="R9" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="S9" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="T9" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="U9" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="V9" t="s">
         <v>56</v>
       </c>
       <c r="W9" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="X9" t="s">
-        <v>145</v>
+        <v>98</v>
       </c>
       <c r="Y9" t="s">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="Z9" t="s">
-        <v>154</v>
+        <v>96</v>
       </c>
       <c r="AA9" t="s">
-        <v>61</v>
+        <v>161</v>
       </c>
       <c r="AB9" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="AC9" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="AD9" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="AE9" t="s">
         <v>65</v>
       </c>
       <c r="AF9" t="s">
-        <v>108</v>
+        <v>66</v>
       </c>
       <c r="AG9" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="AH9" t="s">
-        <v>68</v>
+        <v>164</v>
       </c>
       <c r="AI9" t="s">
-        <v>69</v>
+        <v>165</v>
       </c>
       <c r="AJ9" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="AK9" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="AL9" t="s">
-        <v>113</v>
+        <v>150</v>
       </c>
       <c r="AM9" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.3">
@@ -2605,118 +2845,118 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>84</v>
+        <v>169</v>
       </c>
       <c r="E10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
         <v>44</v>
       </c>
       <c r="G10" t="s">
-        <v>183</v>
+        <v>44</v>
       </c>
       <c r="H10" t="s">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="I10" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="J10" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="K10" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="L10" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="M10" t="s">
-        <v>50</v>
+        <v>135</v>
       </c>
       <c r="N10" t="s">
-        <v>100</v>
+        <v>173</v>
       </c>
       <c r="O10" t="s">
-        <v>101</v>
+        <v>174</v>
       </c>
       <c r="P10" t="s">
-        <v>44</v>
+        <v>175</v>
       </c>
       <c r="Q10" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="R10" t="s">
-        <v>189</v>
+        <v>139</v>
       </c>
       <c r="S10" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="T10" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="U10" t="s">
-        <v>82</v>
+        <v>142</v>
       </c>
       <c r="V10" t="s">
         <v>56</v>
       </c>
       <c r="W10" t="s">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="X10" t="s">
-        <v>190</v>
+        <v>98</v>
       </c>
       <c r="Y10" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="Z10" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="AA10" t="s">
-        <v>61</v>
+        <v>177</v>
       </c>
       <c r="AB10" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="AC10" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="AD10" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="AE10" t="s">
         <v>65</v>
       </c>
       <c r="AF10" t="s">
-        <v>128</v>
+        <v>68</v>
       </c>
       <c r="AG10" t="s">
-        <v>192</v>
+        <v>179</v>
       </c>
       <c r="AH10" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
       <c r="AI10" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="AJ10" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="AK10" t="s">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="AL10" t="s">
-        <v>113</v>
+        <v>150</v>
       </c>
       <c r="AM10" t="s">
-        <v>44</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.3">
@@ -2724,13 +2964,13 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>84</v>
+        <v>183</v>
       </c>
       <c r="E11" t="s">
         <v>43</v>
@@ -2739,102 +2979,816 @@
         <v>44</v>
       </c>
       <c r="G11" t="s">
-        <v>183</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="I11" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="J11" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="K11" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="L11" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="M11" t="s">
         <v>50</v>
       </c>
       <c r="N11" t="s">
-        <v>199</v>
+        <v>77</v>
       </c>
       <c r="O11" t="s">
-        <v>200</v>
+        <v>78</v>
       </c>
       <c r="P11" t="s">
-        <v>201</v>
+        <v>44</v>
       </c>
       <c r="Q11" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="R11" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="S11" t="s">
-        <v>80</v>
+        <v>190</v>
       </c>
       <c r="T11" t="s">
-        <v>204</v>
+        <v>191</v>
       </c>
       <c r="U11" t="s">
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="V11" t="s">
         <v>56</v>
       </c>
       <c r="W11" t="s">
-        <v>83</v>
+        <v>193</v>
       </c>
       <c r="X11" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
       <c r="Y11" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="Z11" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="AA11" t="s">
-        <v>84</v>
+        <v>127</v>
       </c>
       <c r="AB11" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
       <c r="AC11" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
       <c r="AD11" t="s">
-        <v>208</v>
+        <v>98</v>
       </c>
       <c r="AE11" t="s">
         <v>65</v>
       </c>
       <c r="AF11" t="s">
+        <v>196</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>98</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>197</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>198</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>83</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>200</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" t="s">
+        <v>203</v>
+      </c>
+      <c r="F12" t="s">
+        <v>203</v>
+      </c>
+      <c r="G12" t="s">
+        <v>204</v>
+      </c>
+      <c r="H12" t="s">
+        <v>205</v>
+      </c>
+      <c r="I12" t="s">
+        <v>107</v>
+      </c>
+      <c r="J12" t="s">
+        <v>206</v>
+      </c>
+      <c r="K12" t="s">
+        <v>207</v>
+      </c>
+      <c r="L12" t="s">
+        <v>208</v>
+      </c>
+      <c r="M12" t="s">
+        <v>50</v>
+      </c>
+      <c r="N12" t="s">
+        <v>77</v>
+      </c>
+      <c r="O12" t="s">
+        <v>78</v>
+      </c>
+      <c r="P12" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q12" t="s">
         <v>209</v>
       </c>
-      <c r="AG11" t="s">
+      <c r="R12" t="s">
         <v>210</v>
       </c>
-      <c r="AH11" t="s">
-        <v>91</v>
-      </c>
-      <c r="AI11" t="s">
+      <c r="S12" t="s">
+        <v>140</v>
+      </c>
+      <c r="T12" t="s">
+        <v>141</v>
+      </c>
+      <c r="U12" t="s">
+        <v>142</v>
+      </c>
+      <c r="V12" t="s">
+        <v>56</v>
+      </c>
+      <c r="W12" t="s">
+        <v>143</v>
+      </c>
+      <c r="X12" t="s">
         <v>211</v>
       </c>
-      <c r="AJ11" t="s">
-        <v>91</v>
-      </c>
-      <c r="AK11" t="s">
+      <c r="Y12" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z12" t="s">
         <v>212</v>
       </c>
-      <c r="AL11" t="s">
+      <c r="AA12" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB12" t="s">
         <v>213</v>
       </c>
-      <c r="AM11" t="s">
+      <c r="AC12" t="s">
+        <v>213</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>214</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>215</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>216</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>164</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>165</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK12" t="s">
+        <v>217</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>150</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>98</v>
+      </c>
+      <c r="E13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" t="s">
+        <v>88</v>
+      </c>
+      <c r="H13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I13" t="s">
+        <v>220</v>
+      </c>
+      <c r="J13" t="s">
+        <v>221</v>
+      </c>
+      <c r="K13" t="s">
+        <v>222</v>
+      </c>
+      <c r="L13" t="s">
+        <v>223</v>
+      </c>
+      <c r="M13" t="s">
+        <v>50</v>
+      </c>
+      <c r="N13" t="s">
+        <v>77</v>
+      </c>
+      <c r="O13" t="s">
+        <v>78</v>
+      </c>
+      <c r="P13" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>224</v>
+      </c>
+      <c r="R13" t="s">
+        <v>225</v>
+      </c>
+      <c r="S13" t="s">
+        <v>140</v>
+      </c>
+      <c r="T13" t="s">
+        <v>141</v>
+      </c>
+      <c r="U13" t="s">
+        <v>142</v>
+      </c>
+      <c r="V13" t="s">
+        <v>56</v>
+      </c>
+      <c r="W13" t="s">
+        <v>143</v>
+      </c>
+      <c r="X13" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>143</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>143</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>226</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>227</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>228</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>229</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>230</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>231</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>150</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>232</v>
+      </c>
+      <c r="C14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" t="s">
+        <v>203</v>
+      </c>
+      <c r="F14" t="s">
+        <v>203</v>
+      </c>
+      <c r="G14" t="s">
+        <v>204</v>
+      </c>
+      <c r="H14" t="s">
+        <v>205</v>
+      </c>
+      <c r="I14" t="s">
+        <v>233</v>
+      </c>
+      <c r="J14" t="s">
+        <v>234</v>
+      </c>
+      <c r="K14" t="s">
+        <v>235</v>
+      </c>
+      <c r="L14" t="s">
+        <v>236</v>
+      </c>
+      <c r="M14" t="s">
+        <v>50</v>
+      </c>
+      <c r="N14" t="s">
+        <v>77</v>
+      </c>
+      <c r="O14" t="s">
+        <v>78</v>
+      </c>
+      <c r="P14" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>238</v>
+      </c>
+      <c r="R14" t="s">
+        <v>239</v>
+      </c>
+      <c r="S14" t="s">
+        <v>140</v>
+      </c>
+      <c r="T14" t="s">
+        <v>141</v>
+      </c>
+      <c r="U14" t="s">
+        <v>142</v>
+      </c>
+      <c r="V14" t="s">
+        <v>56</v>
+      </c>
+      <c r="W14" t="s">
+        <v>143</v>
+      </c>
+      <c r="X14" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>212</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>213</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>213</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>214</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>215</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>216</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>69</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>240</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>241</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>242</v>
+      </c>
+      <c r="C15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E15" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" t="s">
+        <v>243</v>
+      </c>
+      <c r="H15" t="s">
+        <v>244</v>
+      </c>
+      <c r="I15" t="s">
+        <v>155</v>
+      </c>
+      <c r="J15" t="s">
+        <v>245</v>
+      </c>
+      <c r="K15" t="s">
+        <v>246</v>
+      </c>
+      <c r="L15" t="s">
+        <v>247</v>
+      </c>
+      <c r="M15" t="s">
+        <v>50</v>
+      </c>
+      <c r="N15" t="s">
+        <v>77</v>
+      </c>
+      <c r="O15" t="s">
+        <v>78</v>
+      </c>
+      <c r="P15" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>248</v>
+      </c>
+      <c r="R15" t="s">
+        <v>249</v>
+      </c>
+      <c r="S15" t="s">
+        <v>140</v>
+      </c>
+      <c r="T15" t="s">
+        <v>141</v>
+      </c>
+      <c r="U15" t="s">
+        <v>142</v>
+      </c>
+      <c r="V15" t="s">
+        <v>56</v>
+      </c>
+      <c r="W15" t="s">
+        <v>143</v>
+      </c>
+      <c r="X15" t="s">
+        <v>250</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>212</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>213</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>213</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>251</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>125</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>252</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK15" t="s">
+        <v>253</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>241</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>254</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" t="s">
+        <v>169</v>
+      </c>
+      <c r="E16" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" t="s">
+        <v>131</v>
+      </c>
+      <c r="I16" t="s">
+        <v>255</v>
+      </c>
+      <c r="J16" t="s">
+        <v>256</v>
+      </c>
+      <c r="K16" t="s">
+        <v>257</v>
+      </c>
+      <c r="L16" t="s">
+        <v>258</v>
+      </c>
+      <c r="M16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N16" t="s">
+        <v>77</v>
+      </c>
+      <c r="O16" t="s">
+        <v>78</v>
+      </c>
+      <c r="P16" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>260</v>
+      </c>
+      <c r="R16" t="s">
+        <v>261</v>
+      </c>
+      <c r="S16" t="s">
+        <v>140</v>
+      </c>
+      <c r="T16" t="s">
+        <v>141</v>
+      </c>
+      <c r="U16" t="s">
+        <v>142</v>
+      </c>
+      <c r="V16" t="s">
+        <v>56</v>
+      </c>
+      <c r="W16" t="s">
+        <v>143</v>
+      </c>
+      <c r="X16" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>98</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>262</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>263</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>264</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>264</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>264</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>215</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>265</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>266</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>267</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK16" t="s">
+        <v>268</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>241</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="17" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" t="s">
+        <v>270</v>
+      </c>
+      <c r="C17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" t="s">
+        <v>243</v>
+      </c>
+      <c r="H17" t="s">
+        <v>271</v>
+      </c>
+      <c r="I17" t="s">
+        <v>155</v>
+      </c>
+      <c r="J17" t="s">
+        <v>272</v>
+      </c>
+      <c r="K17" t="s">
+        <v>273</v>
+      </c>
+      <c r="L17" t="s">
+        <v>274</v>
+      </c>
+      <c r="M17" t="s">
+        <v>50</v>
+      </c>
+      <c r="N17" t="s">
+        <v>275</v>
+      </c>
+      <c r="O17" t="s">
+        <v>276</v>
+      </c>
+      <c r="P17" t="s">
+        <v>277</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>278</v>
+      </c>
+      <c r="R17" t="s">
+        <v>279</v>
+      </c>
+      <c r="S17" t="s">
+        <v>140</v>
+      </c>
+      <c r="T17" t="s">
+        <v>280</v>
+      </c>
+      <c r="U17" t="s">
+        <v>281</v>
+      </c>
+      <c r="V17" t="s">
+        <v>56</v>
+      </c>
+      <c r="W17" t="s">
+        <v>143</v>
+      </c>
+      <c r="X17" t="s">
+        <v>282</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>283</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>98</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>143</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>143</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>284</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>285</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>286</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>148</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>287</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>148</v>
+      </c>
+      <c r="AK17" t="s">
+        <v>288</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>289</v>
+      </c>
+      <c r="AM17" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>